<commit_message>
saving after sending draft
</commit_message>
<xml_diff>
--- a/results/Color_lmm_model_results.xlsx
+++ b/results/Color_lmm_model_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madelynore/Documents/Cornell/BTBW_geographic_coloration/BTBW_plumage/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{242276FD-CD47-DB47-AC63-8C7337BB9F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4AEC36D-8CA7-9444-816D-1F6D5BDBB200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="700" windowWidth="26740" windowHeight="15500" xr2:uid="{D5AF6178-8750-6C44-86E9-82514936D21E}"/>
+    <workbookView xWindow="140" yWindow="700" windowWidth="26740" windowHeight="15460" xr2:uid="{48B26526-FCE9-944E-81BE-C027FEADC3A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Color_lmm_model_results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
   <si>
     <t>Response</t>
   </si>
@@ -31,41 +31,38 @@
     <t>Crown PC1</t>
   </si>
   <si>
-    <t>Wing spot PC1</t>
+    <t>~Dorsum PC1 + (1|Year) + (1|preparator)</t>
   </si>
   <si>
-    <t>Wing spot area (mm2)</t>
+    <t>Covert PC1</t>
+  </si>
+  <si>
+    <t>Belly PC1</t>
   </si>
   <si>
     <t>Throat PC1</t>
   </si>
   <si>
-    <t>Coverts PC1</t>
+    <t>~Wing spot PC1 + (1|Year) + (1|preparator)</t>
   </si>
   <si>
-    <t>Belly PC1</t>
+    <t>Dorsum PC1</t>
   </si>
   <si>
-    <t>marginal R2</t>
+    <t>~Wing spot area + (1|Year) + (1|preparator)</t>
   </si>
   <si>
-    <t>P-value</t>
+    <t>Rm2</t>
   </si>
   <si>
-    <t>Dorsum PC1 + (1| Year) + (1|Preparator)</t>
-  </si>
-  <si>
-    <t>Throat PC1  + (1| Year) + (1|Preparator)</t>
+    <t>P value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="0.0000"/>
-  </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -196,12 +193,6 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -548,18 +539,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -610,7 +595,20 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -939,14 +937,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C962B28F-0D90-F24D-86BA-A3509C3677EB}">
-  <dimension ref="A1:D9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3881E36C-E788-B74B-AFAD-A0A244381ECC}">
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.5" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="4" width="18.5" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="38.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -957,118 +954,197 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="3">
-        <v>0.20777024388963</v>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.20799999999999999</v>
       </c>
       <c r="D2" s="2">
-        <v>5.6932395314814496E-7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+        <v>5.6899999999999997E-7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="3">
-        <v>6.6184422319747804E-2</v>
+        <v>4</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="1">
+        <v>0.25900000000000001</v>
       </c>
       <c r="D3" s="2">
-        <v>6.0575900944092797E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+        <v>2.67E-7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="1">
+        <v>0.112</v>
+      </c>
+      <c r="D5" s="2">
+        <v>8.6700000000000004E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2.7E-2</v>
+      </c>
+      <c r="D6" s="1">
+        <v>6.7000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="3">
-        <v>1.4626461194247799E-3</v>
-      </c>
-      <c r="D4" s="4">
-        <v>0.66939569694547696</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="1">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="3">
-        <v>0.112465857273815</v>
-      </c>
-      <c r="D5" s="2">
-        <v>8.66756383604784E-4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="B8" s="3"/>
+      <c r="C8" s="1">
+        <v>1.4E-2</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="1">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="D9" s="1">
+        <v>8.9999999999999993E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="3">
-        <v>0.25879581191908202</v>
-      </c>
-      <c r="D6" s="2">
-        <v>2.6713329645475301E-7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="3">
-        <v>1.0271721016557199E-2</v>
-      </c>
-      <c r="D7" s="4">
-        <v>0.28999999999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="3">
-        <v>3.6569253892461198E-2</v>
-      </c>
-      <c r="D8" s="4">
-        <v>4.7414743885589299E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="D10" s="1">
+        <v>6.5000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1.13E-4</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.90600000000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="3">
-        <v>2.5956743838922301E-3</v>
-      </c>
-      <c r="D9" s="4">
-        <v>0.57157004362998098</v>
+      <c r="B12" s="3"/>
+      <c r="C12" s="1">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0.47299999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="1">
+        <v>2E-3</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="2">
+        <v>2.5399999999999999E-4</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0.82299999999999995</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.70699999999999996</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:B7"/>
-    <mergeCell ref="B8:B9"/>
+  <mergeCells count="3">
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="B11:B15"/>
   </mergeCells>
-  <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <conditionalFormatting sqref="D2:D15">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThanOrEqual">
+      <formula>0.05</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>